<commit_message>
Pay tables from the primary source; engineering and method standard
Minimums are now rebuilt to the cent from Confcommercio's operating note of
29 March 2024 (tables at 1 March 2025 plus the art. 213 increases per tranche).
The secondary sources used before were wrong in three places: Quadri lacked
260.76 EUR of other elements, contingency for Quadri, levels 1 and 2 was off
by one or two cents, level 6 in February 2027 by one cent. Data and results
regenerated; the November tranche totals move by one or two cents.

The INPS rounding rule (F10) now cites the UniEmens technical document,
v4.33 of 29 September 2026.

Also: ruff and return types in CI, coverage in the run summary, pre-commit;
docs/decisioni.md and docs/dizionario-dati.md, kept complete by a test; the
English summary moves to the top of the README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/foglio_controllo_cedolini.xlsx
+++ b/deliverables/foglio_controllo_cedolini.xlsx
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="D14" s="30" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="E14" s="31">
         <f>Mese!X11</f>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="D20" s="30" t="n">
-        <v>1970.29</v>
+        <v>1970.28</v>
       </c>
       <c r="E20" s="31">
         <f>Mese!AG11</f>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="D28" s="30" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="E28" s="31">
         <f>Mese!X23</f>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="D34" s="30" t="n">
-        <v>1752.09</v>
+        <v>1752.08</v>
       </c>
       <c r="E34" s="31">
         <f>Mese!AG23</f>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="D63" s="30" t="n">
-        <v>2723.45</v>
+        <v>2984.22</v>
       </c>
       <c r="E63" s="31">
         <f>Mese!X53</f>
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="D66" s="30" t="n">
-        <v>257.32</v>
+        <v>281.31</v>
       </c>
       <c r="E66" s="31">
         <f>Mese!AB53</f>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="D67" s="30" t="n">
-        <v>241.96</v>
+        <v>264.5</v>
       </c>
       <c r="E67" s="31">
         <f>Mese!AC53</f>
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="D69" s="30" t="n">
-        <v>2009.89</v>
+        <v>2155.51</v>
       </c>
       <c r="E69" s="31">
         <f>Mese!AG53</f>
@@ -4232,7 +4232,7 @@
         </is>
       </c>
       <c r="D126" s="30" t="n">
-        <v>1675.2</v>
+        <v>1675.19</v>
       </c>
       <c r="E126" s="31">
         <f>Mese!X107</f>
@@ -4394,7 +4394,7 @@
         </is>
       </c>
       <c r="D132" s="30" t="n">
-        <v>1347.19</v>
+        <v>1347.18</v>
       </c>
       <c r="E132" s="31">
         <f>Mese!AG107</f>
@@ -9889,7 +9889,7 @@
         </is>
       </c>
       <c r="D325" s="30" t="n">
-        <v>2558.81</v>
+        <v>2558.8</v>
       </c>
       <c r="E325" s="31">
         <f>'Novembre 2026'!J30</f>
@@ -10213,7 +10213,7 @@
         </is>
       </c>
       <c r="D337" s="30" t="n">
-        <v>2280.95</v>
+        <v>2280.93</v>
       </c>
       <c r="E337" s="31">
         <f>'Novembre 2026'!J45</f>
@@ -10753,7 +10753,7 @@
         </is>
       </c>
       <c r="D357" s="30" t="n">
-        <v>2280.95</v>
+        <v>2280.93</v>
       </c>
       <c r="E357" s="31">
         <f>'Novembre 2026'!J70</f>
@@ -12832,7 +12832,7 @@
         </is>
       </c>
       <c r="D434" s="30" t="n">
-        <v>2492.17</v>
+        <v>2492.16</v>
       </c>
       <c r="E434" s="31">
         <f>Riepilogo!D20</f>
@@ -12859,7 +12859,7 @@
         </is>
       </c>
       <c r="D435" s="30" t="n">
-        <v>869.9400000000001</v>
+        <v>869.9299999999999</v>
       </c>
       <c r="E435" s="31">
         <f>Riepilogo!E20</f>
@@ -12940,7 +12940,7 @@
         </is>
       </c>
       <c r="D438" s="30" t="n">
-        <v>303.62</v>
+        <v>303.61</v>
       </c>
       <c r="E438" s="31">
         <f>Riepilogo!E21</f>
@@ -12994,7 +12994,7 @@
         </is>
       </c>
       <c r="D440" s="30" t="n">
-        <v>1594.74</v>
+        <v>1594.73</v>
       </c>
       <c r="E440" s="31">
         <f>Riepilogo!D22</f>
@@ -14929,7 +14929,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="J11" s="15" t="n">
         <v>1</v>
@@ -14944,13 +14944,13 @@
         <v>0</v>
       </c>
       <c r="N11" s="17" t="n">
-        <v>2728.91</v>
+        <v>2728.9</v>
       </c>
       <c r="O11" s="17" t="n">
         <v>250.8</v>
       </c>
       <c r="P11" s="17" t="n">
-        <v>2478.11</v>
+        <v>2478.1</v>
       </c>
       <c r="Q11" s="17" t="n">
         <v>470.65</v>
@@ -14959,7 +14959,7 @@
         <v>37.17</v>
       </c>
       <c r="S11" s="17" t="n">
-        <v>1970.29</v>
+        <v>1970.28</v>
       </c>
       <c r="T11" s="17" t="n">
         <v>235.83</v>
@@ -16957,7 +16957,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="J23" s="15" t="n">
         <v>6</v>
@@ -16972,22 +16972,22 @@
         <v>0</v>
       </c>
       <c r="N23" s="17" t="n">
-        <v>2370.58</v>
+        <v>2370.56</v>
       </c>
       <c r="O23" s="17" t="n">
         <v>217.89</v>
       </c>
       <c r="P23" s="17" t="n">
-        <v>2152.69</v>
+        <v>2152.67</v>
       </c>
       <c r="Q23" s="17" t="n">
-        <v>368.31</v>
+        <v>368.3</v>
       </c>
       <c r="R23" s="17" t="n">
         <v>32.29</v>
       </c>
       <c r="S23" s="17" t="n">
-        <v>1752.09</v>
+        <v>1752.08</v>
       </c>
       <c r="T23" s="17" t="n">
         <v>204.86</v>
@@ -17126,7 +17126,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="J24" s="15" t="n">
         <v>9</v>
@@ -17141,13 +17141,13 @@
         <v>0</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>2727.63</v>
+        <v>2727.62</v>
       </c>
       <c r="O24" s="17" t="n">
         <v>250.7</v>
       </c>
       <c r="P24" s="17" t="n">
-        <v>2476.93</v>
+        <v>2476.92</v>
       </c>
       <c r="Q24" s="17" t="n">
         <v>470.21</v>
@@ -17156,7 +17156,7 @@
         <v>37.15</v>
       </c>
       <c r="S24" s="17" t="n">
-        <v>1969.57</v>
+        <v>1969.56</v>
       </c>
       <c r="T24" s="17" t="n">
         <v>235.72</v>
@@ -17637,7 +17637,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="J27" s="15" t="n">
         <v>6</v>
@@ -17652,13 +17652,13 @@
         <v>0</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>2490.58</v>
+        <v>2490.56</v>
       </c>
       <c r="O27" s="17" t="n">
         <v>228.92</v>
       </c>
       <c r="P27" s="17" t="n">
-        <v>2261.66</v>
+        <v>2261.64</v>
       </c>
       <c r="Q27" s="17" t="n">
         <v>397.73</v>
@@ -17667,10 +17667,10 @@
         <v>33.92</v>
       </c>
       <c r="S27" s="17" t="n">
-        <v>1830.01</v>
+        <v>1829.99</v>
       </c>
       <c r="T27" s="17" t="n">
-        <v>215.24</v>
+        <v>215.23</v>
       </c>
       <c r="U27" s="18" t="n">
         <v>2.1667</v>
@@ -18144,7 +18144,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="J30" s="15" t="n">
         <v>3</v>
@@ -18159,13 +18159,13 @@
         <v>0</v>
       </c>
       <c r="N30" s="17" t="n">
-        <v>2628.59</v>
+        <v>2628.58</v>
       </c>
       <c r="O30" s="17" t="n">
         <v>241.61</v>
       </c>
       <c r="P30" s="17" t="n">
-        <v>2386.98</v>
+        <v>2386.97</v>
       </c>
       <c r="Q30" s="17" t="n">
         <v>436.93</v>
@@ -18174,7 +18174,7 @@
         <v>35.8</v>
       </c>
       <c r="S30" s="17" t="n">
-        <v>1914.25</v>
+        <v>1914.24</v>
       </c>
       <c r="T30" s="17" t="n">
         <v>227.16</v>
@@ -20679,7 +20679,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="17" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="J45" s="15" t="n">
         <v>6</v>
@@ -20694,13 +20694,13 @@
         <v>0</v>
       </c>
       <c r="N45" s="17" t="n">
-        <v>2670.58</v>
+        <v>2670.56</v>
       </c>
       <c r="O45" s="17" t="n">
         <v>245.46</v>
       </c>
       <c r="P45" s="17" t="n">
-        <v>2425.12</v>
+        <v>2425.1</v>
       </c>
       <c r="Q45" s="17" t="n">
         <v>451.04</v>
@@ -20709,7 +20709,7 @@
         <v>36.38</v>
       </c>
       <c r="S45" s="17" t="n">
-        <v>1937.7</v>
+        <v>1937.68</v>
       </c>
       <c r="T45" s="17" t="n">
         <v>230.79</v>
@@ -21186,7 +21186,7 @@
         <v>1</v>
       </c>
       <c r="I48" s="17" t="n">
-        <v>2186.25</v>
+        <v>2186.23</v>
       </c>
       <c r="J48" s="15" t="n">
         <v>4</v>
@@ -21201,22 +21201,22 @@
         <v>0</v>
       </c>
       <c r="N48" s="17" t="n">
-        <v>2577.57</v>
+        <v>2577.55</v>
       </c>
       <c r="O48" s="17" t="n">
         <v>236.92</v>
       </c>
       <c r="P48" s="17" t="n">
-        <v>2340.65</v>
+        <v>2340.63</v>
       </c>
       <c r="Q48" s="17" t="n">
-        <v>419.79</v>
+        <v>419.78</v>
       </c>
       <c r="R48" s="17" t="n">
         <v>35.11</v>
       </c>
       <c r="S48" s="17" t="n">
-        <v>1885.75</v>
+        <v>1885.74</v>
       </c>
       <c r="T48" s="17" t="n">
         <v>222.75</v>
@@ -21693,7 +21693,7 @@
         <v>1</v>
       </c>
       <c r="I51" s="17" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="J51" s="15" t="n">
         <v>0</v>
@@ -21708,13 +21708,13 @@
         <v>0</v>
       </c>
       <c r="N51" s="17" t="n">
-        <v>2584.07</v>
+        <v>2584.06</v>
       </c>
       <c r="O51" s="17" t="n">
         <v>237.47</v>
       </c>
       <c r="P51" s="17" t="n">
-        <v>2346.6</v>
+        <v>2346.59</v>
       </c>
       <c r="Q51" s="17" t="n">
         <v>421.99</v>
@@ -21723,7 +21723,7 @@
         <v>35.2</v>
       </c>
       <c r="S51" s="17" t="n">
-        <v>1889.41</v>
+        <v>1889.4</v>
       </c>
       <c r="T51" s="17" t="n">
         <v>223.31</v>
@@ -22031,7 +22031,7 @@
         <v>1</v>
       </c>
       <c r="I53" s="17" t="n">
-        <v>2723.45</v>
+        <v>2984.22</v>
       </c>
       <c r="J53" s="15" t="n">
         <v>3</v>
@@ -22046,25 +22046,25 @@
         <v>0</v>
       </c>
       <c r="N53" s="17" t="n">
-        <v>2799.83</v>
+        <v>3060.6</v>
       </c>
       <c r="O53" s="17" t="n">
-        <v>257.32</v>
+        <v>281.31</v>
       </c>
       <c r="P53" s="17" t="n">
-        <v>2542.51</v>
+        <v>2779.29</v>
       </c>
       <c r="Q53" s="17" t="n">
-        <v>494.48</v>
+        <v>582.09</v>
       </c>
       <c r="R53" s="17" t="n">
-        <v>38.14</v>
+        <v>41.69</v>
       </c>
       <c r="S53" s="17" t="n">
-        <v>2009.89</v>
+        <v>2155.51</v>
       </c>
       <c r="T53" s="17" t="n">
-        <v>241.96</v>
+        <v>264.5</v>
       </c>
       <c r="U53" s="18" t="n">
         <v>2.1667</v>
@@ -24908,7 +24908,7 @@
         <v>1</v>
       </c>
       <c r="I70" s="17" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="J70" s="15" t="n">
         <v>2</v>
@@ -24923,13 +24923,13 @@
         <v>0</v>
       </c>
       <c r="N70" s="17" t="n">
-        <v>2279.26</v>
+        <v>2279.24</v>
       </c>
       <c r="O70" s="17" t="n">
         <v>209.44</v>
       </c>
       <c r="P70" s="17" t="n">
-        <v>2069.82</v>
+        <v>2069.8</v>
       </c>
       <c r="Q70" s="17" t="n">
         <v>345.93</v>
@@ -24938,7 +24938,7 @@
         <v>31.05</v>
       </c>
       <c r="S70" s="17" t="n">
-        <v>1692.84</v>
+        <v>1692.82</v>
       </c>
       <c r="T70" s="17" t="n">
         <v>196.97</v>
@@ -26940,7 +26940,7 @@
         <v>1</v>
       </c>
       <c r="I82" s="17" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="J82" s="15" t="n">
         <v>1</v>
@@ -26955,13 +26955,13 @@
         <v>0</v>
       </c>
       <c r="N82" s="17" t="n">
-        <v>2728.91</v>
+        <v>2728.9</v>
       </c>
       <c r="O82" s="17" t="n">
         <v>250.8</v>
       </c>
       <c r="P82" s="17" t="n">
-        <v>2478.11</v>
+        <v>2478.1</v>
       </c>
       <c r="Q82" s="17" t="n">
         <v>470.65</v>
@@ -26970,7 +26970,7 @@
         <v>37.17</v>
       </c>
       <c r="S82" s="17" t="n">
-        <v>1970.29</v>
+        <v>1970.28</v>
       </c>
       <c r="T82" s="17" t="n">
         <v>235.83</v>
@@ -28968,7 +28968,7 @@
         <v>1</v>
       </c>
       <c r="I94" s="17" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="J94" s="15" t="n">
         <v>7</v>
@@ -28983,22 +28983,22 @@
         <v>1059.83</v>
       </c>
       <c r="N94" s="17" t="n">
-        <v>3453.24</v>
+        <v>3453.22</v>
       </c>
       <c r="O94" s="17" t="n">
         <v>317.33</v>
       </c>
       <c r="P94" s="17" t="n">
-        <v>3135.91</v>
+        <v>3135.89</v>
       </c>
       <c r="Q94" s="17" t="n">
-        <v>714.04</v>
+        <v>714.03</v>
       </c>
       <c r="R94" s="17" t="n">
         <v>47.04</v>
       </c>
       <c r="S94" s="17" t="n">
-        <v>2374.83</v>
+        <v>2374.82</v>
       </c>
       <c r="T94" s="17" t="n">
         <v>206.84</v>
@@ -31165,7 +31165,7 @@
         <v>1</v>
       </c>
       <c r="I107" s="17" t="n">
-        <v>1675.2</v>
+        <v>1675.19</v>
       </c>
       <c r="J107" s="15" t="n">
         <v>2</v>
@@ -31180,13 +31180,13 @@
         <v>0</v>
       </c>
       <c r="N107" s="17" t="n">
-        <v>1746.95</v>
+        <v>1746.94</v>
       </c>
       <c r="O107" s="17" t="n">
         <v>160.55</v>
       </c>
       <c r="P107" s="17" t="n">
-        <v>1586.4</v>
+        <v>1586.39</v>
       </c>
       <c r="Q107" s="17" t="n">
         <v>215.41</v>
@@ -31195,7 +31195,7 @@
         <v>23.8</v>
       </c>
       <c r="S107" s="17" t="n">
-        <v>1347.19</v>
+        <v>1347.18</v>
       </c>
       <c r="T107" s="17" t="n">
         <v>150.97</v>
@@ -31503,7 +31503,7 @@
         <v>1</v>
       </c>
       <c r="I109" s="17" t="n">
-        <v>2723.45</v>
+        <v>2984.22</v>
       </c>
       <c r="J109" s="15" t="n">
         <v>1</v>
@@ -31518,25 +31518,25 @@
         <v>0</v>
       </c>
       <c r="N109" s="17" t="n">
-        <v>3048.91</v>
+        <v>3309.68</v>
       </c>
       <c r="O109" s="17" t="n">
-        <v>280.2</v>
+        <v>304.19</v>
       </c>
       <c r="P109" s="17" t="n">
-        <v>2768.71</v>
+        <v>3005.49</v>
       </c>
       <c r="Q109" s="17" t="n">
-        <v>578.17</v>
+        <v>665.78</v>
       </c>
       <c r="R109" s="17" t="n">
-        <v>41.53</v>
+        <v>45.08</v>
       </c>
       <c r="S109" s="17" t="n">
-        <v>2149.01</v>
+        <v>2294.63</v>
       </c>
       <c r="T109" s="17" t="n">
-        <v>263.49</v>
+        <v>286.02</v>
       </c>
       <c r="U109" s="18" t="n">
         <v>2.1667</v>
@@ -46855,7 +46855,7 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>1970.29</v>
+        <v>1970.28</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>17.3519</v>
@@ -47239,7 +47239,7 @@
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1752.09</v>
+        <v>1752.08</v>
       </c>
       <c r="D23" s="18" t="n">
         <v>20.113</v>
@@ -47271,7 +47271,7 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1969.57</v>
+        <v>1969.56</v>
       </c>
       <c r="D24" s="18" t="n">
         <v>7.9673</v>
@@ -47367,7 +47367,7 @@
         </is>
       </c>
       <c r="C27" s="17" t="n">
-        <v>1830.01</v>
+        <v>1829.99</v>
       </c>
       <c r="D27" s="18" t="n">
         <v>20.5321</v>
@@ -47463,7 +47463,7 @@
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>1914.25</v>
+        <v>1914.24</v>
       </c>
       <c r="D30" s="18" t="n">
         <v>17.7804</v>
@@ -47943,7 +47943,7 @@
         </is>
       </c>
       <c r="C45" s="17" t="n">
-        <v>1937.7</v>
+        <v>1937.68</v>
       </c>
       <c r="D45" s="18" t="n">
         <v>9.230600000000001</v>
@@ -48039,7 +48039,7 @@
         </is>
       </c>
       <c r="C48" s="17" t="n">
-        <v>1899.48</v>
+        <v>1899.47</v>
       </c>
       <c r="D48" s="18" t="n">
         <v>4.6458</v>
@@ -48135,7 +48135,7 @@
         </is>
       </c>
       <c r="C51" s="17" t="n">
-        <v>1889.41</v>
+        <v>1889.4</v>
       </c>
       <c r="D51" s="18" t="n">
         <v>5.2692</v>
@@ -48199,7 +48199,7 @@
         </is>
       </c>
       <c r="C53" s="17" t="n">
-        <v>2009.89</v>
+        <v>2155.51</v>
       </c>
       <c r="D53" s="18" t="n">
         <v>11.5295</v>
@@ -48743,7 +48743,7 @@
         </is>
       </c>
       <c r="C70" s="17" t="n">
-        <v>1692.84</v>
+        <v>1692.82</v>
       </c>
       <c r="D70" s="18" t="n">
         <v>9.1441</v>
@@ -49127,7 +49127,7 @@
         </is>
       </c>
       <c r="C82" s="17" t="n">
-        <v>1970.29</v>
+        <v>1970.28</v>
       </c>
       <c r="D82" s="18" t="n">
         <v>12.1962</v>
@@ -49511,7 +49511,7 @@
         </is>
       </c>
       <c r="C94" s="17" t="n">
-        <v>1752.09</v>
+        <v>1752.08</v>
       </c>
       <c r="D94" s="18" t="n">
         <v>5.922</v>
@@ -49991,7 +49991,7 @@
         </is>
       </c>
       <c r="C109" s="17" t="n">
-        <v>2149.01</v>
+        <v>2294.63</v>
       </c>
       <c r="D109" s="18" t="n">
         <v>21.9779</v>
@@ -50581,7 +50581,7 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>17977</v>
+        <v>18064.58</v>
       </c>
       <c r="C6" s="19">
         <f>ROUND(SUMIFS(Mese!$Q$5:$Q$254,Mese!$B$5:$B$254,A6),2)</f>
@@ -50592,7 +50592,7 @@
         <v/>
       </c>
       <c r="E6" s="17" t="n">
-        <v>12763.85</v>
+        <v>12787.84</v>
       </c>
       <c r="F6" s="19">
         <f>ROUND(SUMIFS(Mese!$O$5:$O$254,Mese!$B$5:$B$254,A6),2)</f>
@@ -50614,7 +50614,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>6045.7</v>
+        <v>6133.31</v>
       </c>
       <c r="C7" s="19">
         <f>ROUND(SUMIFS(Mese!$Q$5:$Q$254,Mese!$B$5:$B$254,A7),2)</f>
@@ -50625,7 +50625,7 @@
         <v/>
       </c>
       <c r="E7" s="17" t="n">
-        <v>4462.36</v>
+        <v>4486.35</v>
       </c>
       <c r="F7" s="19">
         <f>ROUND(SUMIFS(Mese!$O$5:$O$254,Mese!$B$5:$B$254,A7),2)</f>
@@ -62344,22 +62344,22 @@
         <v>2183.09</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>540.36</v>
+        <v>540.37</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>0</v>
+        <v>260.76</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>2662.68</v>
+        <v>2923.46</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>2723.45</v>
+        <v>2984.22</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>2784.22</v>
+        <v>3044.98</v>
       </c>
       <c r="H5" s="17" t="n">
-        <v>2853.66</v>
+        <v>3114.42</v>
       </c>
       <c r="I5" s="17" t="n">
         <v>25.46</v>
@@ -62375,19 +62375,19 @@
         <v>1966.54</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>537.53</v>
+        <v>537.52</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>2449.33</v>
+        <v>2449.32</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>2504.07</v>
+        <v>2504.06</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>2558.81</v>
+        <v>2558.8</v>
       </c>
       <c r="H6" s="17" t="n">
         <v>2621.36</v>
@@ -62406,22 +62406,22 @@
         <v>1701.04</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>532.5599999999999</v>
+        <v>532.54</v>
       </c>
       <c r="D7" s="17" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>2186.25</v>
+        <v>2186.23</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>2233.6</v>
+        <v>2233.58</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>2280.95</v>
+        <v>2280.93</v>
       </c>
       <c r="H7" s="17" t="n">
-        <v>2335.06</v>
+        <v>2335.04</v>
       </c>
       <c r="I7" s="17" t="n">
         <v>22.83</v>
@@ -62545,7 +62545,7 @@
         <v>1568.09</v>
       </c>
       <c r="H11" s="17" t="n">
-        <v>1600.54</v>
+        <v>1600.53</v>
       </c>
       <c r="I11" s="17" t="n">
         <v>19.73</v>

</xml_diff>